<commit_message>
Add F-column label style for boxed vertical chronology text.
Support displayStyle=label for goal_design-like filled vertical labels, refresh the template with mixed visual patterns, and document the new column contract.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="レーン1" sheetId="1" r:id="rId1"/>
-    <sheet name="レーン2" sheetId="2" r:id="rId2"/>
-    <sheet name="レーン3" sheetId="3" r:id="rId3"/>
-    <sheet name="レーン4" sheetId="4" r:id="rId4"/>
-    <sheet name="レーン5" sheetId="5" r:id="rId5"/>
+    <sheet name="1_点テキスト" sheetId="1" r:id="rId1"/>
+    <sheet name="2_期間バー" sheetId="2" r:id="rId2"/>
+    <sheet name="3_ラベルボックス" sheetId="3" r:id="rId3"/>
+    <sheet name="4_混在パターン" sheetId="4" r:id="rId4"/>
+    <sheet name="5_境界値" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -401,13 +401,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F8"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,70 +427,119 @@
       <c r="E1" t="str">
         <v>色</v>
       </c>
+      <c r="F1" t="str">
+        <v>表示スタイル</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
         <v>1900</v>
       </c>
       <c r="C2" t="str">
-        <v>テスト発生</v>
-      </c>
-      <c r="E2" t="str">
-        <v>#1565C0</v>
+        <v>デフォルト黒文字</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1950</v>
+        <v>1920</v>
       </c>
       <c r="C3" t="str">
-        <v>テスト中</v>
-      </c>
-      <c r="D3">
-        <v>14</v>
+        <v>青い文字</v>
       </c>
       <c r="E3" t="str">
-        <v>#C45C26</v>
+        <v>#1565C0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2000</v>
+        <v>1940</v>
       </c>
       <c r="C4" t="str">
-        <v>テスト確認</v>
+        <v>大きい赤字</v>
+      </c>
+      <c r="D4">
+        <v>16</v>
+      </c>
+      <c r="E4" t="str">
+        <v>#B33A3A</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>2025</v>
+        <v>1960</v>
       </c>
       <c r="C5" t="str">
-        <v>テスト成功</v>
+        <v>小さい紫</v>
       </c>
       <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5" t="str">
+        <v>#5B4B8A</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1985</v>
+      </c>
+      <c r="C6" t="str">
+        <v>緑14px</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#2E7D32</v>
+      </c>
+      <c r="F6" t="str">
+        <v>text</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>2000</v>
+      </c>
+      <c r="C7" t="str">
+        <v>英語 sample</v>
+      </c>
+      <c r="D7">
         <v>12</v>
       </c>
-      <c r="E5" t="str">
-        <v>#1F7A6C</v>
+      <c r="E7" t="str">
+        <v>#E65100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>2015</v>
+      </c>
+      <c r="C8" t="str">
+        <v>あいうえお</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#00838F</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,73 +558,111 @@
       <c r="E1" t="str">
         <v>色</v>
       </c>
+      <c r="F1" t="str">
+        <v>表示スタイル</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1945</v>
+        <v>1910</v>
+      </c>
+      <c r="B2">
+        <v>1925</v>
       </c>
       <c r="C2" t="str">
-        <v>出来事〇〇〇〇</v>
+        <v>短い期間バー</v>
       </c>
       <c r="E2" t="str">
-        <v>#B33A3A</v>
+        <v>#5D4037</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1965</v>
+        <v>1930</v>
+      </c>
+      <c r="B3">
+        <v>1955</v>
       </c>
       <c r="C3" t="str">
-        <v>出来事□□□□</v>
+        <v>中くらいの期間</v>
       </c>
       <c r="D3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="str">
-        <v>#5B4B8A</v>
+        <v>#C45C26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1985</v>
+        <v>1945</v>
       </c>
       <c r="C4" t="str">
-        <v>出来事△△△△</v>
+        <v>点イベント挟み</v>
       </c>
       <c r="E4" t="str">
-        <v>#5D4037</v>
+        <v>#1565C0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>2010</v>
+        <v>1960</v>
+      </c>
+      <c r="B5">
+        <v>1990</v>
       </c>
       <c r="C5" t="str">
-        <v>出来事＋＋＋＋</v>
+        <v>長い期間バー</v>
       </c>
       <c r="D5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E5" t="str">
-        <v>#E65100</v>
+        <v>#1F7A6C</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1970</v>
+      </c>
+      <c r="C6" t="str">
+        <v>重なり確認用の点</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#AD1457</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1995</v>
+      </c>
+      <c r="B7">
+        <v>2005</v>
+      </c>
+      <c r="C7" t="str">
+        <v>短い期間2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#455A64</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -593,56 +681,144 @@
       <c r="E1" t="str">
         <v>色</v>
       </c>
+      <c r="F1" t="str">
+        <v>表示スタイル</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>2000</v>
+        <v>1910</v>
+      </c>
+      <c r="B2">
+        <v>1935</v>
       </c>
       <c r="C2" t="str">
-        <v>あ</v>
+        <v>デモクラシー時代</v>
+      </c>
+      <c r="D2">
+        <v>13</v>
       </c>
       <c r="E2" t="str">
-        <v>#00838F</v>
+        <v>#C45C26</v>
+      </c>
+      <c r="F2" t="str">
+        <v>label</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>2012</v>
+        <v>1920</v>
       </c>
       <c r="C3" t="str">
-        <v>い</v>
+        <v>点は横ボックス</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="str">
-        <v>#AD1457</v>
+        <v>#5B4B8A</v>
+      </c>
+      <c r="F3" t="str">
+        <v>label</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2018</v>
+        <v>1940</v>
+      </c>
+      <c r="B4">
+        <v>1975</v>
       </c>
       <c r="C4" t="str">
-        <v>う</v>
+        <v>高度成長</v>
+      </c>
+      <c r="D4">
+        <v>14</v>
+      </c>
+      <c r="E4" t="str">
+        <v>#1565C0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>1950</v>
+      </c>
+      <c r="B5">
+        <v>1960</v>
+      </c>
+      <c r="C5" t="str">
+        <v>短いラベル</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5" t="str">
+        <v>#1F7A6C</v>
+      </c>
+      <c r="F5" t="str">
+        <v>ラベル</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1970</v>
+      </c>
+      <c r="B6">
+        <v>2000</v>
+      </c>
+      <c r="C6" t="str">
+        <v>バブルへ</v>
+      </c>
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#B33A3A</v>
+      </c>
+      <c r="F6" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1985</v>
+      </c>
+      <c r="B7">
+        <v>1995</v>
+      </c>
+      <c r="C7" t="str">
+        <v>カラー試験</v>
+      </c>
+      <c r="D7">
+        <v>12</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#E65100</v>
+      </c>
+      <c r="F7" t="str">
+        <v>label</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -661,73 +837,154 @@
       <c r="E1" t="str">
         <v>色</v>
       </c>
+      <c r="F1" t="str">
+        <v>表示スタイル</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1958</v>
+        <v>1900</v>
       </c>
       <c r="C2" t="str">
-        <v>aaaa</v>
+        <v>通常テキスト</v>
       </c>
       <c r="E2" t="str">
-        <v>#C2185B</v>
+        <v>#000000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>2000</v>
+        <v>1910</v>
+      </c>
+      <c r="B3">
+        <v>1940</v>
       </c>
       <c r="C3" t="str">
-        <v>bbbb</v>
+        <v>ラベル期間</v>
       </c>
       <c r="D3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" t="str">
-        <v>#2E7D32</v>
+        <v>#5B4B8A</v>
+      </c>
+      <c r="F3" t="str">
+        <v>label</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2005</v>
+        <v>1925</v>
       </c>
       <c r="C4" t="str">
-        <v>cccc</v>
+        <v>色付き点</v>
       </c>
       <c r="E4" t="str">
-        <v>#455A64</v>
+        <v>#C2185B</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>2017</v>
+        <v>1935</v>
+      </c>
+      <c r="B5">
+        <v>1955</v>
       </c>
       <c r="C5" t="str">
-        <v>dddd</v>
-      </c>
-      <c r="D5">
+        <v>期間バー</v>
+      </c>
+      <c r="E5" t="str">
+        <v>#2E7D32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1950</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ラベル点</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#00838F</v>
+      </c>
+      <c r="F6" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1960</v>
+      </c>
+      <c r="B7">
+        <v>1990</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ラベル長期間</v>
+      </c>
+      <c r="D7">
+        <v>14</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#1565C0</v>
+      </c>
+      <c r="F7" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>1975</v>
+      </c>
+      <c r="C8" t="str">
+        <v>大きい文字</v>
+      </c>
+      <c r="D8">
+        <v>18</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#E65100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1988</v>
+      </c>
+      <c r="B9">
+        <v>2000</v>
+      </c>
+      <c r="C9" t="str">
+        <v>バー短め</v>
+      </c>
+      <c r="D9">
         <v>11</v>
       </c>
-      <c r="E5" t="str">
-        <v>#6A1B9A</v>
+      <c r="E9" t="str">
+        <v>#5D4037</v>
+      </c>
+      <c r="F9" t="str">
+        <v>default</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -746,41 +1003,47 @@
       <c r="E1" t="str">
         <v>色</v>
       </c>
+      <c r="F1" t="str">
+        <v>表示スタイル</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1934</v>
+        <v>1900</v>
       </c>
       <c r="C2" t="str">
-        <v>eeee</v>
+        <v>最小フォント</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
+      </c>
+      <c r="E2" t="str">
+        <v>#37474F</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1955</v>
+        <v>1910</v>
       </c>
       <c r="C3" t="str">
-        <v>ffff</v>
+        <v>最大フォント</v>
       </c>
       <c r="D3">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="E3" t="str">
-        <v>#EF6C00</v>
+        <v>#B33A3A</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1956</v>
+        <v>1920</v>
       </c>
       <c r="B4">
-        <v>1998</v>
+        <v>1921</v>
       </c>
       <c r="C4" t="str">
-        <v>gggg</v>
-      </c>
-      <c r="D4">
-        <v>14</v>
+        <v>1年だけ期間</v>
       </c>
       <c r="E4" t="str">
         <v>#1565C0</v>
@@ -788,18 +1051,89 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>1966</v>
+        <v>1930</v>
+      </c>
+      <c r="B5">
+        <v>1931</v>
       </c>
       <c r="C5" t="str">
-        <v>hhhh</v>
+        <v>1年ラベル</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
       </c>
       <c r="E5" t="str">
-        <v>#37474F</v>
+        <v>#C45C26</v>
+      </c>
+      <c r="F5" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>1940</v>
+      </c>
+      <c r="C6" t="str">
+        <v>RGB指定</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6" t="str">
+        <v>rgb(21,101,192)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1950</v>
+      </c>
+      <c r="C7" t="str">
+        <v>3桁色</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#F0A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>1960</v>
+      </c>
+      <c r="B8">
+        <v>1990</v>
+      </c>
+      <c r="C8" t="str">
+        <v>長いラベルボックス文言テスト</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#6A1B9A</v>
+      </c>
+      <c r="F8" t="str">
+        <v>label</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1980</v>
+      </c>
+      <c r="C9" t="str">
+        <v>無効スタイルは無視</v>
+      </c>
+      <c r="D9">
+        <v>11</v>
+      </c>
+      <c r="E9" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="F9" t="str">
+        <v>box</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>